<commit_message>
Move broker, distributor, and sales commission fees under A&P section
The three new $/case fees now live at Inputs rows 115-117 directly
below Royalties, rather than appended after the freight section.
Freight per pallet section shifts to rows 119-124; Freight Model
formulas and the P&L by Scenario formulas are retargeted to the new
input row positions. Properly shifts merged ranges across the
insertion point so no cell data is lost.

https://claude.ai/code/session_01Hq85TUVVzULd2nbqwzzsbG
</commit_message>
<xml_diff>
--- a/RTD_PL_updated.xlsx
+++ b/RTD_PL_updated.xlsx
@@ -3957,137 +3957,138 @@
         <v>0</v>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>Broker fees</t>
+        </is>
+      </c>
+      <c r="B115" s="18" t="inlineStr">
+        <is>
+          <t>$/case</t>
+        </is>
+      </c>
+      <c r="D115" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E115" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F115" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G115" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H115" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I115" s="32" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
     <row r="116" ht="15" customHeight="1">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>Freight per pallet</t>
-        </is>
+      <c r="A116" s="15" t="inlineStr">
+        <is>
+          <t>Distributor fees</t>
+        </is>
+      </c>
+      <c r="B116" s="18" t="inlineStr">
+        <is>
+          <t>$/case</t>
+        </is>
+      </c>
+      <c r="D116" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E116" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F116" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G116" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H116" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I116" s="32" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="15" t="inlineStr">
         <is>
-          <t>Inbound rate</t>
+          <t>Sales team commission</t>
         </is>
       </c>
       <c r="B117" s="18" t="inlineStr">
         <is>
-          <t>$/pallet</t>
-        </is>
-      </c>
-      <c r="D117" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="E117" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="F117" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="G117" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="H117" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="I117" s="33" t="n">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="15" t="inlineStr">
-        <is>
-          <t>Transfer rate, DC to DC</t>
-        </is>
-      </c>
-      <c r="B118" s="18" t="inlineStr">
-        <is>
-          <t>$/pallet</t>
-        </is>
-      </c>
-      <c r="D118" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E118" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F118" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G118" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H118" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I118" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
+          <t>$/case</t>
+        </is>
+      </c>
+      <c r="D117" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E117" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F117" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G117" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H117" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I117" s="32" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="118"/>
     <row r="119">
-      <c r="A119" s="15" t="inlineStr">
-        <is>
-          <t>Outbound rate</t>
-        </is>
-      </c>
-      <c r="B119" s="18" t="inlineStr">
-        <is>
-          <t>$/pallet</t>
-        </is>
-      </c>
-      <c r="D119" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="E119" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="F119" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="G119" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="H119" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="I119" s="33" t="n">
-        <v>250</v>
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Freight per pallet</t>
+        </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="15" t="inlineStr">
         <is>
-          <t>Fuel surcharge</t>
+          <t>Inbound rate</t>
         </is>
       </c>
       <c r="B120" s="18" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D120" s="24" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E120" s="24" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F120" s="24" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="G120" s="24" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H120" s="24" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I120" s="24" t="n">
-        <v>0.15</v>
+          <t>$/pallet</t>
+        </is>
+      </c>
+      <c r="D120" s="33" t="n">
+        <v>250</v>
+      </c>
+      <c r="E120" s="33" t="n">
+        <v>250</v>
+      </c>
+      <c r="F120" s="33" t="n">
+        <v>250</v>
+      </c>
+      <c r="G120" s="33" t="n">
+        <v>250</v>
+      </c>
+      <c r="H120" s="33" t="n">
+        <v>250</v>
+      </c>
+      <c r="I120" s="33" t="n">
+        <v>250</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="15" t="inlineStr">
         <is>
-          <t>LTL premium per pallet</t>
+          <t>Transfer rate, DC to DC</t>
         </is>
       </c>
       <c r="B121" s="18" t="inlineStr">
@@ -4096,112 +4097,112 @@
         </is>
       </c>
       <c r="D121" s="33" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E121" s="33" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F121" s="33" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="G121" s="33" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="H121" s="33" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="I121" s="33" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="15" t="inlineStr">
         <is>
-          <t>Broker fees</t>
+          <t>Outbound rate</t>
         </is>
       </c>
       <c r="B122" s="18" t="inlineStr">
         <is>
-          <t>$/case</t>
-        </is>
-      </c>
-      <c r="D122" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E122" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F122" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G122" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H122" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I122" s="32" t="n">
-        <v>0.5</v>
+          <t>$/pallet</t>
+        </is>
+      </c>
+      <c r="D122" s="33" t="n">
+        <v>250</v>
+      </c>
+      <c r="E122" s="33" t="n">
+        <v>250</v>
+      </c>
+      <c r="F122" s="33" t="n">
+        <v>250</v>
+      </c>
+      <c r="G122" s="33" t="n">
+        <v>250</v>
+      </c>
+      <c r="H122" s="33" t="n">
+        <v>250</v>
+      </c>
+      <c r="I122" s="33" t="n">
+        <v>250</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="15" t="inlineStr">
         <is>
-          <t>Distributor fees</t>
+          <t>Fuel surcharge</t>
         </is>
       </c>
       <c r="B123" s="18" t="inlineStr">
         <is>
-          <t>$/case</t>
-        </is>
-      </c>
-      <c r="D123" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E123" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="F123" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G123" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="H123" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="I123" s="32" t="n">
-        <v>1</v>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D123" s="24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E123" s="24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F123" s="24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G123" s="24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H123" s="24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I123" s="24" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="15" t="inlineStr">
         <is>
-          <t>Sales team commission</t>
+          <t>LTL premium per pallet</t>
         </is>
       </c>
       <c r="B124" s="18" t="inlineStr">
         <is>
-          <t>$/case</t>
-        </is>
-      </c>
-      <c r="D124" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E124" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F124" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G124" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H124" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I124" s="32" t="n">
-        <v>0.5</v>
+          <t>$/pallet</t>
+        </is>
+      </c>
+      <c r="D124" s="33" t="n">
+        <v>50</v>
+      </c>
+      <c r="E124" s="33" t="n">
+        <v>50</v>
+      </c>
+      <c r="F124" s="33" t="n">
+        <v>50</v>
+      </c>
+      <c r="G124" s="33" t="n">
+        <v>50</v>
+      </c>
+      <c r="H124" s="33" t="n">
+        <v>50</v>
+      </c>
+      <c r="I124" s="33" t="n">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -4214,7 +4215,6 @@
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A47:I47"/>
     <mergeCell ref="A14:I14"/>
-    <mergeCell ref="A116:I116"/>
     <mergeCell ref="A91:I91"/>
     <mergeCell ref="A20:I20"/>
     <mergeCell ref="A38:I38"/>
@@ -4227,6 +4227,7 @@
     <mergeCell ref="A107:I107"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A70:I70"/>
+    <mergeCell ref="A119:I119"/>
     <mergeCell ref="A69:I69"/>
     <mergeCell ref="A87:I87"/>
     <mergeCell ref="A78:I78"/>
@@ -6872,27 +6873,27 @@
         </is>
       </c>
       <c r="D7" s="16">
-        <f>Inputs!D117*(1+Inputs!D120)</f>
+        <f>Inputs!D120*(1+Inputs!D123)</f>
         <v/>
       </c>
       <c r="E7" s="16">
-        <f>Inputs!E117*(1+Inputs!E120)</f>
+        <f>Inputs!E120*(1+Inputs!E123)</f>
         <v/>
       </c>
       <c r="F7" s="16">
-        <f>Inputs!F117*(1+Inputs!F120)</f>
+        <f>Inputs!F120*(1+Inputs!F123)</f>
         <v/>
       </c>
       <c r="G7" s="16">
-        <f>Inputs!G117*(1+Inputs!G120)</f>
+        <f>Inputs!G120*(1+Inputs!G123)</f>
         <v/>
       </c>
       <c r="H7" s="16">
-        <f>Inputs!H117*(1+Inputs!H120)</f>
+        <f>Inputs!H120*(1+Inputs!H123)</f>
         <v/>
       </c>
       <c r="I7" s="16">
-        <f>Inputs!I117*(1+Inputs!I120)</f>
+        <f>Inputs!I120*(1+Inputs!I123)</f>
         <v/>
       </c>
     </row>
@@ -6908,27 +6909,27 @@
         </is>
       </c>
       <c r="D8" s="16">
-        <f>Inputs!D118*(1+Inputs!D120)</f>
+        <f>Inputs!D121*(1+Inputs!D123)</f>
         <v/>
       </c>
       <c r="E8" s="16">
-        <f>Inputs!E118*(1+Inputs!E120)</f>
+        <f>Inputs!E121*(1+Inputs!E123)</f>
         <v/>
       </c>
       <c r="F8" s="16">
-        <f>Inputs!F118*(1+Inputs!F120)</f>
+        <f>Inputs!F121*(1+Inputs!F123)</f>
         <v/>
       </c>
       <c r="G8" s="16">
-        <f>Inputs!G118*(1+Inputs!G120)</f>
+        <f>Inputs!G121*(1+Inputs!G123)</f>
         <v/>
       </c>
       <c r="H8" s="16">
-        <f>Inputs!H118*(1+Inputs!H120)</f>
+        <f>Inputs!H121*(1+Inputs!H123)</f>
         <v/>
       </c>
       <c r="I8" s="16">
-        <f>Inputs!I118*(1+Inputs!I120)</f>
+        <f>Inputs!I121*(1+Inputs!I123)</f>
         <v/>
       </c>
     </row>
@@ -6944,27 +6945,27 @@
         </is>
       </c>
       <c r="D9" s="16">
-        <f>Inputs!D119*(1+Inputs!D120)</f>
+        <f>Inputs!D122*(1+Inputs!D123)</f>
         <v/>
       </c>
       <c r="E9" s="16">
-        <f>Inputs!E119*(1+Inputs!E120)</f>
+        <f>Inputs!E122*(1+Inputs!E123)</f>
         <v/>
       </c>
       <c r="F9" s="16">
-        <f>Inputs!F119*(1+Inputs!F120)</f>
+        <f>Inputs!F122*(1+Inputs!F123)</f>
         <v/>
       </c>
       <c r="G9" s="16">
-        <f>Inputs!G119*(1+Inputs!G120)</f>
+        <f>Inputs!G122*(1+Inputs!G123)</f>
         <v/>
       </c>
       <c r="H9" s="16">
-        <f>Inputs!H119*(1+Inputs!H120)</f>
+        <f>Inputs!H122*(1+Inputs!H123)</f>
         <v/>
       </c>
       <c r="I9" s="16">
-        <f>Inputs!I119*(1+Inputs!I120)</f>
+        <f>Inputs!I122*(1+Inputs!I123)</f>
         <v/>
       </c>
     </row>
@@ -6980,27 +6981,27 @@
         </is>
       </c>
       <c r="D10" s="16">
-        <f>Inputs!D121</f>
+        <f>Inputs!D124</f>
         <v/>
       </c>
       <c r="E10" s="16">
-        <f>Inputs!E121</f>
+        <f>Inputs!E124</f>
         <v/>
       </c>
       <c r="F10" s="16">
-        <f>Inputs!F121</f>
+        <f>Inputs!F124</f>
         <v/>
       </c>
       <c r="G10" s="16">
-        <f>Inputs!G121</f>
+        <f>Inputs!G124</f>
         <v/>
       </c>
       <c r="H10" s="16">
-        <f>Inputs!H121</f>
+        <f>Inputs!H124</f>
         <v/>
       </c>
       <c r="I10" s="16">
-        <f>Inputs!I121</f>
+        <f>Inputs!I124</f>
         <v/>
       </c>
     </row>
@@ -8041,51 +8042,51 @@
         </is>
       </c>
       <c r="D23" s="46">
-        <f>((Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D122+Inputs!D123+Inputs!D124)*Cover!D6</f>
+        <f>((Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D115+Inputs!D116+Inputs!D117)*Cover!D6</f>
         <v/>
       </c>
       <c r="E23" s="46">
-        <f>((Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E122+Inputs!E123+Inputs!E124)*Cover!E6</f>
+        <f>((Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E115+Inputs!E116+Inputs!E117)*Cover!E6</f>
         <v/>
       </c>
       <c r="F23" s="46">
-        <f>((Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F122+Inputs!F123+Inputs!F124)*Cover!F6</f>
+        <f>((Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F115+Inputs!F116+Inputs!F117)*Cover!F6</f>
         <v/>
       </c>
       <c r="G23" s="46">
-        <f>((Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G122+Inputs!G123+Inputs!G124)*Cover!G6</f>
+        <f>((Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G115+Inputs!G116+Inputs!G117)*Cover!G6</f>
         <v/>
       </c>
       <c r="H23" s="46">
-        <f>((Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H122+Inputs!H123+Inputs!H124)*Cover!H6</f>
+        <f>((Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H115+Inputs!H116+Inputs!H117)*Cover!H6</f>
         <v/>
       </c>
       <c r="I23" s="46">
-        <f>((Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I122+Inputs!I123+Inputs!I124)*Cover!I6</f>
+        <f>((Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I115+Inputs!I116+Inputs!I117)*Cover!I6</f>
         <v/>
       </c>
       <c r="K23" s="47">
-        <f>((Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D122+Inputs!D123+Inputs!D124)*Inputs!D10</f>
+        <f>((Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D115+Inputs!D116+Inputs!D117)*Inputs!D10</f>
         <v/>
       </c>
       <c r="L23" s="47">
-        <f>((Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E122+Inputs!E123+Inputs!E124)*Inputs!E10</f>
+        <f>((Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E115+Inputs!E116+Inputs!E117)*Inputs!E10</f>
         <v/>
       </c>
       <c r="M23" s="47">
-        <f>((Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F122+Inputs!F123+Inputs!F124)*Inputs!F10</f>
+        <f>((Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F115+Inputs!F116+Inputs!F117)*Inputs!F10</f>
         <v/>
       </c>
       <c r="N23" s="47">
-        <f>((Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G122+Inputs!G123+Inputs!G124)*Inputs!G10</f>
+        <f>((Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G115+Inputs!G116+Inputs!G117)*Inputs!G10</f>
         <v/>
       </c>
       <c r="O23" s="47">
-        <f>((Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H122+Inputs!H123+Inputs!H124)*Inputs!H10</f>
+        <f>((Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H115+Inputs!H116+Inputs!H117)*Inputs!H10</f>
         <v/>
       </c>
       <c r="P23" s="47">
-        <f>((Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I122+Inputs!I123+Inputs!I124)*Inputs!I10</f>
+        <f>((Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I115+Inputs!I116+Inputs!I117)*Inputs!I10</f>
         <v/>
       </c>
     </row>
@@ -8096,51 +8097,51 @@
         </is>
       </c>
       <c r="D24" s="51">
-        <f>((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124)*Cover!D6</f>
+        <f>((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117)*Cover!D6</f>
         <v/>
       </c>
       <c r="E24" s="51">
-        <f>((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124)*Cover!E6</f>
+        <f>((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117)*Cover!E6</f>
         <v/>
       </c>
       <c r="F24" s="51">
-        <f>((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124)*Cover!F6</f>
+        <f>((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117)*Cover!F6</f>
         <v/>
       </c>
       <c r="G24" s="51">
-        <f>((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124)*Cover!G6</f>
+        <f>((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117)*Cover!G6</f>
         <v/>
       </c>
       <c r="H24" s="51">
-        <f>((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124)*Cover!H6</f>
+        <f>((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117)*Cover!H6</f>
         <v/>
       </c>
       <c r="I24" s="51">
-        <f>((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124)*Cover!I6</f>
+        <f>((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117)*Cover!I6</f>
         <v/>
       </c>
       <c r="K24" s="52">
-        <f>((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124)*Inputs!D10</f>
+        <f>((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117)*Inputs!D10</f>
         <v/>
       </c>
       <c r="L24" s="52">
-        <f>((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124)*Inputs!E10</f>
+        <f>((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117)*Inputs!E10</f>
         <v/>
       </c>
       <c r="M24" s="52">
-        <f>((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124)*Inputs!F10</f>
+        <f>((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117)*Inputs!F10</f>
         <v/>
       </c>
       <c r="N24" s="52">
-        <f>((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124)*Inputs!G10</f>
+        <f>((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117)*Inputs!G10</f>
         <v/>
       </c>
       <c r="O24" s="52">
-        <f>((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124)*Inputs!H10</f>
+        <f>((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117)*Inputs!H10</f>
         <v/>
       </c>
       <c r="P24" s="52">
-        <f>((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124)*Inputs!I10</f>
+        <f>((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117)*Inputs!I10</f>
         <v/>
       </c>
     </row>
@@ -8151,51 +8152,51 @@
         </is>
       </c>
       <c r="D26" s="44">
-        <f>((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124))*Cover!D6</f>
+        <f>((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117))*Cover!D6</f>
         <v/>
       </c>
       <c r="E26" s="44">
-        <f>((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124))*Cover!E6</f>
+        <f>((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117))*Cover!E6</f>
         <v/>
       </c>
       <c r="F26" s="44">
-        <f>((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124))*Cover!F6</f>
+        <f>((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117))*Cover!F6</f>
         <v/>
       </c>
       <c r="G26" s="44">
-        <f>((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124))*Cover!G6</f>
+        <f>((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117))*Cover!G6</f>
         <v/>
       </c>
       <c r="H26" s="44">
-        <f>((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124))*Cover!H6</f>
+        <f>((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117))*Cover!H6</f>
         <v/>
       </c>
       <c r="I26" s="44">
-        <f>((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124))*Cover!I6</f>
+        <f>((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117))*Cover!I6</f>
         <v/>
       </c>
       <c r="K26" s="53">
-        <f>((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124))*Inputs!D10</f>
+        <f>((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117))*Inputs!D10</f>
         <v/>
       </c>
       <c r="L26" s="53">
-        <f>((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124))*Inputs!E10</f>
+        <f>((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117))*Inputs!E10</f>
         <v/>
       </c>
       <c r="M26" s="53">
-        <f>((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124))*Inputs!F10</f>
+        <f>((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117))*Inputs!F10</f>
         <v/>
       </c>
       <c r="N26" s="53">
-        <f>((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124))*Inputs!G10</f>
+        <f>((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117))*Inputs!G10</f>
         <v/>
       </c>
       <c r="O26" s="53">
-        <f>((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124))*Inputs!H10</f>
+        <f>((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117))*Inputs!H10</f>
         <v/>
       </c>
       <c r="P26" s="53">
-        <f>((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124))*Inputs!I10</f>
+        <f>((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117))*Inputs!I10</f>
         <v/>
       </c>
     </row>
@@ -8206,27 +8207,27 @@
         </is>
       </c>
       <c r="D27" s="54">
-        <f>IFERROR(((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124))/(Inputs!D35*(1-Inputs!D44)),0)</f>
+        <f>IFERROR(((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117))/(Inputs!D35*(1-Inputs!D44)),0)</f>
         <v/>
       </c>
       <c r="E27" s="54">
-        <f>IFERROR(((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124))/(Inputs!E35*(1-Inputs!E44)),0)</f>
+        <f>IFERROR(((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117))/(Inputs!E35*(1-Inputs!E44)),0)</f>
         <v/>
       </c>
       <c r="F27" s="54">
-        <f>IFERROR(((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124))/(Inputs!F35*(1-Inputs!F44)),0)</f>
+        <f>IFERROR(((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117))/(Inputs!F35*(1-Inputs!F44)),0)</f>
         <v/>
       </c>
       <c r="G27" s="54">
-        <f>IFERROR(((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124))/(Inputs!G35*(1-Inputs!G44)),0)</f>
+        <f>IFERROR(((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117))/(Inputs!G35*(1-Inputs!G44)),0)</f>
         <v/>
       </c>
       <c r="H27" s="54">
-        <f>IFERROR(((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124))/(Inputs!H35*(1-Inputs!H44)),0)</f>
+        <f>IFERROR(((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117))/(Inputs!H35*(1-Inputs!H44)),0)</f>
         <v/>
       </c>
       <c r="I27" s="54">
-        <f>IFERROR(((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124))/(Inputs!I35*(1-Inputs!I44)),0)</f>
+        <f>IFERROR(((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117))/(Inputs!I35*(1-Inputs!I44)),0)</f>
         <v/>
       </c>
       <c r="K27" s="54">
@@ -8268,51 +8269,51 @@
         </is>
       </c>
       <c r="D30" s="48">
-        <f>(MAX(0,((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124)))*Inputs!D27)*Cover!D6</f>
+        <f>(MAX(0,((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117)))*Inputs!D27)*Cover!D6</f>
         <v/>
       </c>
       <c r="E30" s="48">
-        <f>(MAX(0,((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124)))*Inputs!E27)*Cover!E6</f>
+        <f>(MAX(0,((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117)))*Inputs!E27)*Cover!E6</f>
         <v/>
       </c>
       <c r="F30" s="48">
-        <f>(MAX(0,((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124)))*Inputs!F27)*Cover!F6</f>
+        <f>(MAX(0,((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117)))*Inputs!F27)*Cover!F6</f>
         <v/>
       </c>
       <c r="G30" s="48">
-        <f>(MAX(0,((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124)))*Inputs!G27)*Cover!G6</f>
+        <f>(MAX(0,((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117)))*Inputs!G27)*Cover!G6</f>
         <v/>
       </c>
       <c r="H30" s="48">
-        <f>(MAX(0,((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124)))*Inputs!H27)*Cover!H6</f>
+        <f>(MAX(0,((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117)))*Inputs!H27)*Cover!H6</f>
         <v/>
       </c>
       <c r="I30" s="48">
-        <f>(MAX(0,((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124)))*Inputs!I27)*Cover!I6</f>
+        <f>(MAX(0,((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117)))*Inputs!I27)*Cover!I6</f>
         <v/>
       </c>
       <c r="K30" s="49">
-        <f>(MAX(0,((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124)))*Inputs!D27)*Inputs!D10</f>
+        <f>(MAX(0,((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117)))*Inputs!D27)*Inputs!D10</f>
         <v/>
       </c>
       <c r="L30" s="49">
-        <f>(MAX(0,((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124)))*Inputs!E27)*Inputs!E10</f>
+        <f>(MAX(0,((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117)))*Inputs!E27)*Inputs!E10</f>
         <v/>
       </c>
       <c r="M30" s="49">
-        <f>(MAX(0,((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124)))*Inputs!F27)*Inputs!F10</f>
+        <f>(MAX(0,((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117)))*Inputs!F27)*Inputs!F10</f>
         <v/>
       </c>
       <c r="N30" s="49">
-        <f>(MAX(0,((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124)))*Inputs!G27)*Inputs!G10</f>
+        <f>(MAX(0,((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117)))*Inputs!G27)*Inputs!G10</f>
         <v/>
       </c>
       <c r="O30" s="49">
-        <f>(MAX(0,((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124)))*Inputs!H27)*Inputs!H10</f>
+        <f>(MAX(0,((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117)))*Inputs!H27)*Inputs!H10</f>
         <v/>
       </c>
       <c r="P30" s="49">
-        <f>(MAX(0,((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124)))*Inputs!I27)*Inputs!I10</f>
+        <f>(MAX(0,((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117)))*Inputs!I27)*Inputs!I10</f>
         <v/>
       </c>
     </row>
@@ -8323,51 +8324,51 @@
         </is>
       </c>
       <c r="D31" s="44">
-        <f>(((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124))-MAX(0,((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124)))*Inputs!D27)*Cover!D6</f>
+        <f>(((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117))-MAX(0,((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117)))*Inputs!D27)*Cover!D6</f>
         <v/>
       </c>
       <c r="E31" s="44">
-        <f>(((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124))-MAX(0,((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124)))*Inputs!E27)*Cover!E6</f>
+        <f>(((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117))-MAX(0,((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117)))*Inputs!E27)*Cover!E6</f>
         <v/>
       </c>
       <c r="F31" s="44">
-        <f>(((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124))-MAX(0,((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124)))*Inputs!F27)*Cover!F6</f>
+        <f>(((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117))-MAX(0,((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117)))*Inputs!F27)*Cover!F6</f>
         <v/>
       </c>
       <c r="G31" s="44">
-        <f>(((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124))-MAX(0,((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124)))*Inputs!G27)*Cover!G6</f>
+        <f>(((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117))-MAX(0,((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117)))*Inputs!G27)*Cover!G6</f>
         <v/>
       </c>
       <c r="H31" s="44">
-        <f>(((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124))-MAX(0,((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124)))*Inputs!H27)*Cover!H6</f>
+        <f>(((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117))-MAX(0,((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117)))*Inputs!H27)*Cover!H6</f>
         <v/>
       </c>
       <c r="I31" s="44">
-        <f>(((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124))-MAX(0,((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124)))*Inputs!I27)*Cover!I6</f>
+        <f>(((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117))-MAX(0,((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117)))*Inputs!I27)*Cover!I6</f>
         <v/>
       </c>
       <c r="K31" s="53">
-        <f>(((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124))-MAX(0,((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124)))*Inputs!D27)*Inputs!D10</f>
+        <f>(((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117))-MAX(0,((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117)))*Inputs!D27)*Inputs!D10</f>
         <v/>
       </c>
       <c r="L31" s="53">
-        <f>(((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124))-MAX(0,((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124)))*Inputs!E27)*Inputs!E10</f>
+        <f>(((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117))-MAX(0,((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117)))*Inputs!E27)*Inputs!E10</f>
         <v/>
       </c>
       <c r="M31" s="53">
-        <f>(((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124))-MAX(0,((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124)))*Inputs!F27)*Inputs!F10</f>
+        <f>(((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117))-MAX(0,((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117)))*Inputs!F27)*Inputs!F10</f>
         <v/>
       </c>
       <c r="N31" s="53">
-        <f>(((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124))-MAX(0,((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124)))*Inputs!G27)*Inputs!G10</f>
+        <f>(((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117))-MAX(0,((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117)))*Inputs!G27)*Inputs!G10</f>
         <v/>
       </c>
       <c r="O31" s="53">
-        <f>(((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124))-MAX(0,((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124)))*Inputs!H27)*Inputs!H10</f>
+        <f>(((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117))-MAX(0,((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117)))*Inputs!H27)*Inputs!H10</f>
         <v/>
       </c>
       <c r="P31" s="53">
-        <f>(((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124))-MAX(0,((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124)))*Inputs!I27)*Inputs!I10</f>
+        <f>(((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117))-MAX(0,((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117)))*Inputs!I27)*Inputs!I10</f>
         <v/>
       </c>
     </row>
@@ -8378,27 +8379,27 @@
         </is>
       </c>
       <c r="D32" s="54">
-        <f>IFERROR((((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124))-MAX(0,((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D122+Inputs!D123+Inputs!D124)))*Inputs!D27)/(Inputs!D35*(1-Inputs!D44)),0)</f>
+        <f>IFERROR((((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117))-MAX(0,((Inputs!D35*(1-Inputs!D44))-('Direct COGS'!K39+'Indirect COGS'!K20)-((Inputs!D108+Inputs!D109+Inputs!D110+Inputs!D112+Inputs!D113+Inputs!D114)*(Inputs!D35*(1-Inputs!D44))+Inputs!D111+Inputs!D115+Inputs!D116+Inputs!D117)))*Inputs!D27)/(Inputs!D35*(1-Inputs!D44)),0)</f>
         <v/>
       </c>
       <c r="E32" s="54">
-        <f>IFERROR((((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124))-MAX(0,((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E122+Inputs!E123+Inputs!E124)))*Inputs!E27)/(Inputs!E35*(1-Inputs!E44)),0)</f>
+        <f>IFERROR((((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117))-MAX(0,((Inputs!E35*(1-Inputs!E44))-('Direct COGS'!L39+'Indirect COGS'!L20)-((Inputs!E108+Inputs!E109+Inputs!E110+Inputs!E112+Inputs!E113+Inputs!E114)*(Inputs!E35*(1-Inputs!E44))+Inputs!E111+Inputs!E115+Inputs!E116+Inputs!E117)))*Inputs!E27)/(Inputs!E35*(1-Inputs!E44)),0)</f>
         <v/>
       </c>
       <c r="F32" s="54">
-        <f>IFERROR((((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124))-MAX(0,((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F122+Inputs!F123+Inputs!F124)))*Inputs!F27)/(Inputs!F35*(1-Inputs!F44)),0)</f>
+        <f>IFERROR((((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117))-MAX(0,((Inputs!F35*(1-Inputs!F44))-('Direct COGS'!M39+'Indirect COGS'!M20)-((Inputs!F108+Inputs!F109+Inputs!F110+Inputs!F112+Inputs!F113+Inputs!F114)*(Inputs!F35*(1-Inputs!F44))+Inputs!F111+Inputs!F115+Inputs!F116+Inputs!F117)))*Inputs!F27)/(Inputs!F35*(1-Inputs!F44)),0)</f>
         <v/>
       </c>
       <c r="G32" s="54">
-        <f>IFERROR((((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124))-MAX(0,((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G122+Inputs!G123+Inputs!G124)))*Inputs!G27)/(Inputs!G35*(1-Inputs!G44)),0)</f>
+        <f>IFERROR((((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117))-MAX(0,((Inputs!G35*(1-Inputs!G44))-('Direct COGS'!N39+'Indirect COGS'!N20)-((Inputs!G108+Inputs!G109+Inputs!G110+Inputs!G112+Inputs!G113+Inputs!G114)*(Inputs!G35*(1-Inputs!G44))+Inputs!G111+Inputs!G115+Inputs!G116+Inputs!G117)))*Inputs!G27)/(Inputs!G35*(1-Inputs!G44)),0)</f>
         <v/>
       </c>
       <c r="H32" s="54">
-        <f>IFERROR((((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124))-MAX(0,((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H122+Inputs!H123+Inputs!H124)))*Inputs!H27)/(Inputs!H35*(1-Inputs!H44)),0)</f>
+        <f>IFERROR((((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117))-MAX(0,((Inputs!H35*(1-Inputs!H44))-('Direct COGS'!O39+'Indirect COGS'!O20)-((Inputs!H108+Inputs!H109+Inputs!H110+Inputs!H112+Inputs!H113+Inputs!H114)*(Inputs!H35*(1-Inputs!H44))+Inputs!H111+Inputs!H115+Inputs!H116+Inputs!H117)))*Inputs!H27)/(Inputs!H35*(1-Inputs!H44)),0)</f>
         <v/>
       </c>
       <c r="I32" s="54">
-        <f>IFERROR((((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124))-MAX(0,((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I122+Inputs!I123+Inputs!I124)))*Inputs!I27)/(Inputs!I35*(1-Inputs!I44)),0)</f>
+        <f>IFERROR((((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117))-MAX(0,((Inputs!I35*(1-Inputs!I44))-('Direct COGS'!P39+'Indirect COGS'!P20)-((Inputs!I108+Inputs!I109+Inputs!I110+Inputs!I112+Inputs!I113+Inputs!I114)*(Inputs!I35*(1-Inputs!I44))+Inputs!I111+Inputs!I115+Inputs!I116+Inputs!I117)))*Inputs!I27)/(Inputs!I35*(1-Inputs!I44)),0)</f>
         <v/>
       </c>
       <c r="K32" s="54">

</xml_diff>